<commit_message>
Keep our own bookkeeping out of the reviewer-note column
95 of the 106 notes on report-bound rows were "bulk: B3" / "bulk: B4" — audit
strings the bulk-apply button writes, not reviewer prose. Shipping them would
have put our internal queue codes in a column the library reads as
"reviewer's note". Only the 9 real notes survive.

One of those 9 mixed a question to ourselves ("למה דווח?") with a genuine
finding (a missing closing parenthesis). Sent whole it would open the line by
asking why we reported it. The finding is kept via NOTE_OVERRIDE; the question
stays in decisions.json where it was asked.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/nli-report-20260921.xlsx
+++ b/docs/nli-report-20260921.xlsx
@@ -3694,11 +3694,7 @@
           <t>2892518</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007564322205171</t>
@@ -3751,11 +3747,7 @@
       </c>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007284803205171</t>
@@ -3812,11 +3804,7 @@
           <t>4368319</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007529708805171</t>
@@ -3869,11 +3857,7 @@
       </c>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007555456905171</t>
@@ -3926,11 +3910,7 @@
       </c>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007415889605171</t>
@@ -3983,11 +3963,7 @@
       </c>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007540907105171</t>
@@ -4093,11 +4069,7 @@
       </c>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007554238205171</t>
@@ -4199,11 +4171,7 @@
       </c>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007524670705171</t>
@@ -4317,11 +4285,7 @@
           <t>143160</t>
         </is>
       </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007536434705171</t>
@@ -4435,11 +4399,7 @@
       </c>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007567857705171</t>
@@ -4492,11 +4452,7 @@
       </c>
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007560192505171</t>
@@ -4659,11 +4615,7 @@
           <t>3165250</t>
         </is>
       </c>
-      <c r="L32" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007541762605171</t>
@@ -4769,11 +4721,7 @@
           <t>312116</t>
         </is>
       </c>
-      <c r="L34" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007537927405171</t>
@@ -4883,11 +4831,7 @@
           <t>8953134</t>
         </is>
       </c>
-      <c r="L36" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007550230005171</t>
@@ -4997,11 +4941,7 @@
           <t>6291043</t>
         </is>
       </c>
-      <c r="L38" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007489333905171</t>
@@ -5054,11 +4994,7 @@
       </c>
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007480256305171</t>
@@ -5160,11 +5096,7 @@
       </c>
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007543967105171</t>
@@ -5270,11 +5202,7 @@
       </c>
       <c r="J43" t="inlineStr"/>
       <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007550227305171</t>
@@ -5478,11 +5406,7 @@
       </c>
       <c r="J47" t="inlineStr"/>
       <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L47" t="inlineStr"/>
       <c r="M47" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007529996605171</t>
@@ -5592,11 +5516,7 @@
           <t>2905154</t>
         </is>
       </c>
-      <c r="L49" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L49" t="inlineStr"/>
       <c r="M49" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007564639705171</t>
@@ -5649,11 +5569,7 @@
       </c>
       <c r="J50" t="inlineStr"/>
       <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L50" t="inlineStr"/>
       <c r="M50" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007560553605171</t>
@@ -5710,11 +5626,7 @@
           <t>6071994</t>
         </is>
       </c>
-      <c r="L51" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L51" t="inlineStr"/>
       <c r="M51" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007566381305171</t>
@@ -5767,11 +5679,7 @@
       </c>
       <c r="J52" t="inlineStr"/>
       <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L52" t="inlineStr"/>
       <c r="M52" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007554831505171</t>
@@ -5828,11 +5736,7 @@
           <t>571096</t>
         </is>
       </c>
-      <c r="L53" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L53" t="inlineStr"/>
       <c r="M53" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007534359505171</t>
@@ -5889,11 +5793,7 @@
           <t>2026643</t>
         </is>
       </c>
-      <c r="L54" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L54" t="inlineStr"/>
       <c r="M54" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007554968405171</t>
@@ -5950,11 +5850,7 @@
           <t>3172931</t>
         </is>
       </c>
-      <c r="L55" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L55" t="inlineStr"/>
       <c r="M55" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007564957105171</t>
@@ -6064,11 +5960,7 @@
           <t>11886622</t>
         </is>
       </c>
-      <c r="L57" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L57" t="inlineStr"/>
       <c r="M57" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007562365105171</t>
@@ -6121,11 +6013,7 @@
       </c>
       <c r="J58" t="inlineStr"/>
       <c r="K58" t="inlineStr"/>
-      <c r="L58" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L58" t="inlineStr"/>
       <c r="M58" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007562324405171</t>
@@ -6178,11 +6066,7 @@
       </c>
       <c r="J59" t="inlineStr"/>
       <c r="K59" t="inlineStr"/>
-      <c r="L59" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L59" t="inlineStr"/>
       <c r="M59" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007560013405171</t>
@@ -6235,11 +6119,7 @@
       </c>
       <c r="J60" t="inlineStr"/>
       <c r="K60" t="inlineStr"/>
-      <c r="L60" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L60" t="inlineStr"/>
       <c r="M60" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007564629705171</t>
@@ -6296,11 +6176,7 @@
           <t>627127</t>
         </is>
       </c>
-      <c r="L61" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L61" t="inlineStr"/>
       <c r="M61" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007564905705171</t>
@@ -6459,11 +6335,7 @@
       </c>
       <c r="J64" t="inlineStr"/>
       <c r="K64" t="inlineStr"/>
-      <c r="L64" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L64" t="inlineStr"/>
       <c r="M64" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007564562205171</t>
@@ -6520,11 +6392,7 @@
           <t>2525574</t>
         </is>
       </c>
-      <c r="L65" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L65" t="inlineStr"/>
       <c r="M65" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007564560905171</t>
@@ -6634,11 +6502,7 @@
           <t>757957</t>
         </is>
       </c>
-      <c r="L67" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L67" t="inlineStr"/>
       <c r="M67" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007564939605171</t>
@@ -6691,11 +6555,7 @@
       </c>
       <c r="J68" t="inlineStr"/>
       <c r="K68" t="inlineStr"/>
-      <c r="L68" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L68" t="inlineStr"/>
       <c r="M68" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007564339005171</t>
@@ -6809,11 +6669,7 @@
           <t>3049576</t>
         </is>
       </c>
-      <c r="L70" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L70" t="inlineStr"/>
       <c r="M70" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007562299405171</t>
@@ -6866,11 +6722,7 @@
       </c>
       <c r="J71" t="inlineStr"/>
       <c r="K71" t="inlineStr"/>
-      <c r="L71" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L71" t="inlineStr"/>
       <c r="M71" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007567130205171</t>
@@ -6980,11 +6832,7 @@
       </c>
       <c r="J73" t="inlineStr"/>
       <c r="K73" t="inlineStr"/>
-      <c r="L73" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L73" t="inlineStr"/>
       <c r="M73" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007566950505171</t>
@@ -7143,11 +6991,7 @@
       </c>
       <c r="J76" t="inlineStr"/>
       <c r="K76" t="inlineStr"/>
-      <c r="L76" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L76" t="inlineStr"/>
       <c r="M76" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007560132205171</t>
@@ -7204,11 +7048,7 @@
           <t>759470</t>
         </is>
       </c>
-      <c r="L77" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L77" t="inlineStr"/>
       <c r="M77" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007560004305171</t>
@@ -7367,11 +7207,7 @@
       </c>
       <c r="J80" t="inlineStr"/>
       <c r="K80" t="inlineStr"/>
-      <c r="L80" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L80" t="inlineStr"/>
       <c r="M80" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007567513705171</t>
@@ -7424,11 +7260,7 @@
       </c>
       <c r="J81" t="inlineStr"/>
       <c r="K81" t="inlineStr"/>
-      <c r="L81" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L81" t="inlineStr"/>
       <c r="M81" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007559990305171</t>
@@ -7485,11 +7317,7 @@
           <t>6296382</t>
         </is>
       </c>
-      <c r="L82" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L82" t="inlineStr"/>
       <c r="M82" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007567374905171</t>
@@ -7542,11 +7370,7 @@
       </c>
       <c r="J83" t="inlineStr"/>
       <c r="K83" t="inlineStr"/>
-      <c r="L83" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L83" t="inlineStr"/>
       <c r="M83" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007564435605171</t>
@@ -7599,11 +7423,7 @@
       </c>
       <c r="J84" t="inlineStr"/>
       <c r="K84" t="inlineStr"/>
-      <c r="L84" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L84" t="inlineStr"/>
       <c r="M84" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007564539905171</t>
@@ -7656,11 +7476,7 @@
       </c>
       <c r="J85" t="inlineStr"/>
       <c r="K85" t="inlineStr"/>
-      <c r="L85" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L85" t="inlineStr"/>
       <c r="M85" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007567226805171</t>
@@ -7770,11 +7586,7 @@
           <t>6697805</t>
         </is>
       </c>
-      <c r="L87" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L87" t="inlineStr"/>
       <c r="M87" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007560546705171</t>
@@ -7941,11 +7753,7 @@
           <t>105510</t>
         </is>
       </c>
-      <c r="L90" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L90" t="inlineStr"/>
       <c r="M90" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007561813405171</t>
@@ -7998,11 +7806,7 @@
       </c>
       <c r="J91" t="inlineStr"/>
       <c r="K91" t="inlineStr"/>
-      <c r="L91" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L91" t="inlineStr"/>
       <c r="M91" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007564668505171</t>
@@ -8161,11 +7965,7 @@
       </c>
       <c r="J94" t="inlineStr"/>
       <c r="K94" t="inlineStr"/>
-      <c r="L94" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L94" t="inlineStr"/>
       <c r="M94" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007561828205171</t>
@@ -8275,11 +8075,7 @@
           <t>730435</t>
         </is>
       </c>
-      <c r="L96" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L96" t="inlineStr"/>
       <c r="M96" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007561902705171</t>
@@ -8332,11 +8128,7 @@
       </c>
       <c r="J97" t="inlineStr"/>
       <c r="K97" t="inlineStr"/>
-      <c r="L97" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L97" t="inlineStr"/>
       <c r="M97" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007564798905171</t>
@@ -8442,11 +8234,7 @@
       </c>
       <c r="J99" t="inlineStr"/>
       <c r="K99" t="inlineStr"/>
-      <c r="L99" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L99" t="inlineStr"/>
       <c r="M99" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007560358905171</t>
@@ -8821,11 +8609,7 @@
       </c>
       <c r="J106" t="inlineStr"/>
       <c r="K106" t="inlineStr"/>
-      <c r="L106" t="inlineStr">
-        <is>
-          <t>bulk: B3</t>
-        </is>
-      </c>
+      <c r="L106" t="inlineStr"/>
       <c r="M106" t="inlineStr">
         <is>
           <t>https://www.nli.org.il/he/authorities/987007465731605171</t>
@@ -9905,7 +9689,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>למה דווח? כמו כן  הסוגר הסופי חסר, מה שדורש דיווח לספריה.</t>
+          <t>הסוגר הסופי חסר בכותרת.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr"/>

</xml_diff>